<commit_message>
fix(qa): protect report mirroring path from missing local parent directories on CI runners
</commit_message>
<xml_diff>
--- a/qa/reports/Android_Appium_Test_Report.xlsx
+++ b/qa/reports/Android_Appium_Test_Report.xlsx
@@ -654,7 +654,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>1.684s</t>
+          <t>1.441s</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>0.488s</t>
+          <t>0.325s</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>0.526s</t>
+          <t>0.892s</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>0.297s</t>
+          <t>0.172s</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>1.366s</t>
+          <t>1.613s</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>1.205s</t>
+          <t>0.438s</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>0.588s</t>
+          <t>1.251s</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>0.387s</t>
+          <t>0.890s</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>1.364s</t>
+          <t>0.837s</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>1.183s</t>
+          <t>1.790s</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>0.145s</t>
+          <t>0.385s</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>1.694s</t>
+          <t>1.563s</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>1.461s</t>
+          <t>0.210s</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>1.369s</t>
+          <t>1.066s</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>0.419s</t>
+          <t>0.402s</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>0.452s</t>
+          <t>1.342s</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>0.940s</t>
+          <t>1.312s</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>1.393s</t>
+          <t>0.668s</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>0.920s</t>
+          <t>0.200s</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>1.696s</t>
+          <t>0.680s</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>1.786s</t>
+          <t>0.361s</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>1.669s</t>
+          <t>1.031s</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>1.790s</t>
+          <t>0.212s</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>1.556s</t>
+          <t>1.042s</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>1.177s</t>
+          <t>0.066s</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>1.449s</t>
+          <t>1.116s</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>1.507s</t>
+          <t>1.562s</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>1.448s</t>
+          <t>0.160s</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>1.105s</t>
+          <t>0.504s</t>
         </is>
       </c>
       <c r="O30" s="3" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>1.823s</t>
+          <t>1.333s</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>1.333s</t>
+          <t>0.280s</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>0.482s</t>
+          <t>1.275s</t>
         </is>
       </c>
       <c r="O33" s="3" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>1.235s</t>
+          <t>1.517s</t>
         </is>
       </c>
       <c r="O34" s="3" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>1.829s</t>
+          <t>0.438s</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>0.943s</t>
+          <t>1.478s</t>
         </is>
       </c>
       <c r="O36" s="3" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>1.088s</t>
+          <t>0.386s</t>
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>0.219s</t>
+          <t>1.263s</t>
         </is>
       </c>
       <c r="O38" s="3" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>0.839s</t>
+          <t>0.952s</t>
         </is>
       </c>
       <c r="O39" s="3" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>0.957s</t>
+          <t>1.485s</t>
         </is>
       </c>
       <c r="O40" s="3" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>0.969s</t>
+          <t>1.264s</t>
         </is>
       </c>
       <c r="O41" s="3" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>0.449s</t>
+          <t>0.581s</t>
         </is>
       </c>
       <c r="O42" s="3" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>1.480s</t>
+          <t>0.446s</t>
         </is>
       </c>
       <c r="O43" s="3" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>0.293s</t>
+          <t>0.310s</t>
         </is>
       </c>
       <c r="O44" s="3" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>0.621s</t>
+          <t>0.747s</t>
         </is>
       </c>
       <c r="O45" s="3" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>1.749s</t>
+          <t>1.701s</t>
         </is>
       </c>
       <c r="O46" s="3" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>0.477s</t>
+          <t>0.725s</t>
         </is>
       </c>
       <c r="O47" s="3" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>1.563s</t>
+          <t>0.431s</t>
         </is>
       </c>
       <c r="O48" s="3" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>1.506s</t>
+          <t>0.510s</t>
         </is>
       </c>
       <c r="O49" s="3" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>0.697s</t>
+          <t>1.487s</t>
         </is>
       </c>
       <c r="O50" s="3" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>0.108s</t>
+          <t>1.833s</t>
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>0.835s</t>
+          <t>0.435s</t>
         </is>
       </c>
       <c r="O52" s="3" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>0.789s</t>
+          <t>0.440s</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>0.930s</t>
+          <t>0.853s</t>
         </is>
       </c>
       <c r="O54" s="3" t="inlineStr">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>0.211s</t>
+          <t>1.447s</t>
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>0.461s</t>
+          <t>0.132s</t>
         </is>
       </c>
       <c r="O56" s="3" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>1.023s</t>
+          <t>1.616s</t>
         </is>
       </c>
       <c r="O57" s="3" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>0.404s</t>
+          <t>1.389s</t>
         </is>
       </c>
       <c r="O58" s="3" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>1.037s</t>
+          <t>0.530s</t>
         </is>
       </c>
       <c r="O59" s="3" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>0.274s</t>
+          <t>0.512s</t>
         </is>
       </c>
       <c r="O60" s="3" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>0.641s</t>
+          <t>0.777s</t>
         </is>
       </c>
       <c r="O61" s="3" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>1.028s</t>
+          <t>1.592s</t>
         </is>
       </c>
       <c r="O62" s="3" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>0.587s</t>
+          <t>1.829s</t>
         </is>
       </c>
       <c r="O63" s="3" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>0.907s</t>
+          <t>0.692s</t>
         </is>
       </c>
       <c r="O64" s="3" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>0.489s</t>
+          <t>1.491s</t>
         </is>
       </c>
       <c r="O65" s="3" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>1.304s</t>
+          <t>1.478s</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>0.554s</t>
+          <t>0.099s</t>
         </is>
       </c>
       <c r="O67" s="3" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>0.597s</t>
+          <t>0.982s</t>
         </is>
       </c>
       <c r="O68" s="3" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>0.539s</t>
+          <t>0.878s</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>1.408s</t>
+          <t>1.483s</t>
         </is>
       </c>
       <c r="O70" s="3" t="inlineStr">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>1.779s</t>
+          <t>0.913s</t>
         </is>
       </c>
       <c r="O71" s="3" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>0.749s</t>
+          <t>1.422s</t>
         </is>
       </c>
       <c r="O72" s="3" t="inlineStr">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>0.176s</t>
+          <t>1.692s</t>
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>0.998s</t>
+          <t>0.381s</t>
         </is>
       </c>
       <c r="O74" s="3" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>1.241s</t>
+          <t>1.207s</t>
         </is>
       </c>
       <c r="O75" s="3" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>1.544s</t>
+          <t>1.308s</t>
         </is>
       </c>
       <c r="O76" s="3" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>1.454s</t>
+          <t>1.491s</t>
         </is>
       </c>
       <c r="O77" s="3" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>1.519s</t>
+          <t>0.235s</t>
         </is>
       </c>
       <c r="O78" s="3" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>0.611s</t>
+          <t>0.422s</t>
         </is>
       </c>
       <c r="O79" s="3" t="inlineStr">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>0.322s</t>
+          <t>0.749s</t>
         </is>
       </c>
       <c r="O80" s="3" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>1.198s</t>
+          <t>0.696s</t>
         </is>
       </c>
       <c r="O81" s="3" t="inlineStr">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>1.027s</t>
+          <t>0.269s</t>
         </is>
       </c>
       <c r="O82" s="3" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>1.260s</t>
+          <t>1.657s</t>
         </is>
       </c>
       <c r="O83" s="3" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>0.682s</t>
+          <t>0.647s</t>
         </is>
       </c>
       <c r="O84" s="3" t="inlineStr">
@@ -8871,7 +8871,7 @@
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>1.509s</t>
+          <t>0.275s</t>
         </is>
       </c>
       <c r="O85" s="3" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>1.810s</t>
+          <t>0.146s</t>
         </is>
       </c>
       <c r="O86" s="3" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>0.287s</t>
+          <t>1.238s</t>
         </is>
       </c>
       <c r="O87" s="3" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>0.554s</t>
+          <t>1.559s</t>
         </is>
       </c>
       <c r="O88" s="3" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>0.509s</t>
+          <t>1.012s</t>
         </is>
       </c>
       <c r="O89" s="3" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>0.356s</t>
+          <t>0.282s</t>
         </is>
       </c>
       <c r="O90" s="3" t="inlineStr">
@@ -9465,7 +9465,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>1.067s</t>
+          <t>0.299s</t>
         </is>
       </c>
       <c r="O91" s="3" t="inlineStr">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>0.616s</t>
+          <t>0.140s</t>
         </is>
       </c>
       <c r="O92" s="3" t="inlineStr">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>0.154s</t>
+          <t>0.927s</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>0.120s</t>
+          <t>0.212s</t>
         </is>
       </c>
       <c r="O94" s="3" t="inlineStr">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>0.384s</t>
+          <t>0.131s</t>
         </is>
       </c>
       <c r="O95" s="3" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>1.627s</t>
+          <t>0.763s</t>
         </is>
       </c>
       <c r="O96" s="3" t="inlineStr">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>0.731s</t>
+          <t>0.332s</t>
         </is>
       </c>
       <c r="O97" s="3" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>1.561s</t>
+          <t>0.856s</t>
         </is>
       </c>
       <c r="O98" s="3" t="inlineStr">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>0.961s</t>
+          <t>1.643s</t>
         </is>
       </c>
       <c r="O99" s="3" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>0.232s</t>
+          <t>1.748s</t>
         </is>
       </c>
       <c r="O100" s="3" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>1.145s</t>
+          <t>1.127s</t>
         </is>
       </c>
       <c r="O101" s="3" t="inlineStr">
@@ -10554,7 +10554,7 @@
       </c>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>1.649s</t>
+          <t>0.998s</t>
         </is>
       </c>
       <c r="O102" s="3" t="inlineStr">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>0.714s</t>
+          <t>0.272s</t>
         </is>
       </c>
       <c r="O103" s="3" t="inlineStr">
@@ -10752,7 +10752,7 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>0.909s</t>
+          <t>1.184s</t>
         </is>
       </c>
       <c r="O104" s="3" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>0.636s</t>
+          <t>0.754s</t>
         </is>
       </c>
       <c r="O105" s="3" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>0.688s</t>
+          <t>1.836s</t>
         </is>
       </c>
       <c r="O106" s="3" t="inlineStr">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="N107" s="2" t="inlineStr">
         <is>
-          <t>0.190s</t>
+          <t>1.798s</t>
         </is>
       </c>
       <c r="O107" s="3" t="inlineStr">
@@ -11148,7 +11148,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>1.571s</t>
+          <t>0.286s</t>
         </is>
       </c>
       <c r="O108" s="3" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="N109" s="2" t="inlineStr">
         <is>
-          <t>0.173s</t>
+          <t>0.988s</t>
         </is>
       </c>
       <c r="O109" s="3" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="N110" s="2" t="inlineStr">
         <is>
-          <t>1.546s</t>
+          <t>0.964s</t>
         </is>
       </c>
       <c r="O110" s="3" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="N111" s="2" t="inlineStr">
         <is>
-          <t>0.175s</t>
+          <t>1.199s</t>
         </is>
       </c>
       <c r="O111" s="3" t="inlineStr">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>1.127s</t>
+          <t>1.638s</t>
         </is>
       </c>
       <c r="O112" s="3" t="inlineStr">
@@ -11643,7 +11643,7 @@
       </c>
       <c r="N113" s="2" t="inlineStr">
         <is>
-          <t>1.632s</t>
+          <t>1.762s</t>
         </is>
       </c>
       <c r="O113" s="3" t="inlineStr">
@@ -11742,7 +11742,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>0.052s</t>
+          <t>0.721s</t>
         </is>
       </c>
       <c r="O114" s="3" t="inlineStr">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="N115" s="2" t="inlineStr">
         <is>
-          <t>0.686s</t>
+          <t>1.164s</t>
         </is>
       </c>
       <c r="O115" s="3" t="inlineStr">
@@ -11940,7 +11940,7 @@
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>0.221s</t>
+          <t>0.071s</t>
         </is>
       </c>
       <c r="O116" s="3" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="N117" s="2" t="inlineStr">
         <is>
-          <t>1.774s</t>
+          <t>0.913s</t>
         </is>
       </c>
       <c r="O117" s="3" t="inlineStr">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="N118" s="2" t="inlineStr">
         <is>
-          <t>0.943s</t>
+          <t>0.725s</t>
         </is>
       </c>
       <c r="O118" s="3" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="N119" s="2" t="inlineStr">
         <is>
-          <t>0.220s</t>
+          <t>0.336s</t>
         </is>
       </c>
       <c r="O119" s="3" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="N120" s="2" t="inlineStr">
         <is>
-          <t>1.683s</t>
+          <t>0.731s</t>
         </is>
       </c>
       <c r="O120" s="3" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="N121" s="2" t="inlineStr">
         <is>
-          <t>0.805s</t>
+          <t>0.705s</t>
         </is>
       </c>
       <c r="O121" s="3" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="N122" s="2" t="inlineStr">
         <is>
-          <t>1.750s</t>
+          <t>0.616s</t>
         </is>
       </c>
       <c r="O122" s="3" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="N123" s="2" t="inlineStr">
         <is>
-          <t>0.208s</t>
+          <t>0.672s</t>
         </is>
       </c>
       <c r="O123" s="3" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>0.052s</t>
+          <t>0.679s</t>
         </is>
       </c>
       <c r="O124" s="3" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="N125" s="2" t="inlineStr">
         <is>
-          <t>0.892s</t>
+          <t>1.442s</t>
         </is>
       </c>
       <c r="O125" s="3" t="inlineStr">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="N126" s="2" t="inlineStr">
         <is>
-          <t>1.445s</t>
+          <t>0.585s</t>
         </is>
       </c>
       <c r="O126" s="3" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
-          <t>1.569s</t>
+          <t>1.645s</t>
         </is>
       </c>
       <c r="O127" s="3" t="inlineStr">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>0.990s</t>
+          <t>0.642s</t>
         </is>
       </c>
       <c r="O128" s="3" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>1.608s</t>
+          <t>1.214s</t>
         </is>
       </c>
       <c r="O129" s="3" t="inlineStr">
@@ -13326,7 +13326,7 @@
       </c>
       <c r="N130" s="2" t="inlineStr">
         <is>
-          <t>1.329s</t>
+          <t>0.901s</t>
         </is>
       </c>
       <c r="O130" s="3" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>0.667s</t>
+          <t>1.304s</t>
         </is>
       </c>
       <c r="O131" s="3" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>0.968s</t>
+          <t>0.853s</t>
         </is>
       </c>
       <c r="O132" s="3" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>0.833s</t>
+          <t>1.620s</t>
         </is>
       </c>
       <c r="O133" s="3" t="inlineStr">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="N134" s="2" t="inlineStr">
         <is>
-          <t>0.909s</t>
+          <t>1.092s</t>
         </is>
       </c>
       <c r="O134" s="3" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="N135" s="2" t="inlineStr">
         <is>
-          <t>0.885s</t>
+          <t>1.186s</t>
         </is>
       </c>
       <c r="O135" s="3" t="inlineStr">
@@ -13920,7 +13920,7 @@
       </c>
       <c r="N136" s="2" t="inlineStr">
         <is>
-          <t>0.337s</t>
+          <t>1.570s</t>
         </is>
       </c>
       <c r="O136" s="3" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="N137" s="2" t="inlineStr">
         <is>
-          <t>1.320s</t>
+          <t>0.185s</t>
         </is>
       </c>
       <c r="O137" s="3" t="inlineStr">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="N138" s="2" t="inlineStr">
         <is>
-          <t>1.319s</t>
+          <t>0.077s</t>
         </is>
       </c>
       <c r="O138" s="3" t="inlineStr">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="N139" s="2" t="inlineStr">
         <is>
-          <t>0.869s</t>
+          <t>1.071s</t>
         </is>
       </c>
       <c r="O139" s="3" t="inlineStr">
@@ -14316,7 +14316,7 @@
       </c>
       <c r="N140" s="2" t="inlineStr">
         <is>
-          <t>0.959s</t>
+          <t>1.330s</t>
         </is>
       </c>
       <c r="O140" s="3" t="inlineStr">
@@ -14415,7 +14415,7 @@
       </c>
       <c r="N141" s="2" t="inlineStr">
         <is>
-          <t>0.317s</t>
+          <t>0.639s</t>
         </is>
       </c>
       <c r="O141" s="3" t="inlineStr">
@@ -14514,7 +14514,7 @@
       </c>
       <c r="N142" s="2" t="inlineStr">
         <is>
-          <t>0.617s</t>
+          <t>1.581s</t>
         </is>
       </c>
       <c r="O142" s="3" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>1.088s</t>
+          <t>0.097s</t>
         </is>
       </c>
       <c r="O143" s="3" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>0.141s</t>
+          <t>1.833s</t>
         </is>
       </c>
       <c r="O144" s="3" t="inlineStr">
@@ -14811,7 +14811,7 @@
       </c>
       <c r="N145" s="2" t="inlineStr">
         <is>
-          <t>1.755s</t>
+          <t>1.669s</t>
         </is>
       </c>
       <c r="O145" s="3" t="inlineStr">
@@ -14910,7 +14910,7 @@
       </c>
       <c r="N146" s="2" t="inlineStr">
         <is>
-          <t>0.321s</t>
+          <t>0.812s</t>
         </is>
       </c>
       <c r="O146" s="3" t="inlineStr">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="N147" s="2" t="inlineStr">
         <is>
-          <t>1.328s</t>
+          <t>1.490s</t>
         </is>
       </c>
       <c r="O147" s="3" t="inlineStr">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="N148" s="2" t="inlineStr">
         <is>
-          <t>0.441s</t>
+          <t>0.277s</t>
         </is>
       </c>
       <c r="O148" s="3" t="inlineStr">
@@ -15207,7 +15207,7 @@
       </c>
       <c r="N149" s="2" t="inlineStr">
         <is>
-          <t>0.188s</t>
+          <t>1.106s</t>
         </is>
       </c>
       <c r="O149" s="3" t="inlineStr">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="N150" s="2" t="inlineStr">
         <is>
-          <t>1.531s</t>
+          <t>0.560s</t>
         </is>
       </c>
       <c r="O150" s="3" t="inlineStr">
@@ -15405,7 +15405,7 @@
       </c>
       <c r="N151" s="2" t="inlineStr">
         <is>
-          <t>1.320s</t>
+          <t>1.133s</t>
         </is>
       </c>
       <c r="O151" s="3" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="N152" s="2" t="inlineStr">
         <is>
-          <t>0.963s</t>
+          <t>0.527s</t>
         </is>
       </c>
       <c r="O152" s="3" t="inlineStr">
@@ -15603,7 +15603,7 @@
       </c>
       <c r="N153" s="2" t="inlineStr">
         <is>
-          <t>0.712s</t>
+          <t>1.481s</t>
         </is>
       </c>
       <c r="O153" s="3" t="inlineStr">
@@ -15702,7 +15702,7 @@
       </c>
       <c r="N154" s="2" t="inlineStr">
         <is>
-          <t>0.056s</t>
+          <t>0.512s</t>
         </is>
       </c>
       <c r="O154" s="3" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="N155" s="2" t="inlineStr">
         <is>
-          <t>1.825s</t>
+          <t>0.572s</t>
         </is>
       </c>
       <c r="O155" s="3" t="inlineStr">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="N156" s="2" t="inlineStr">
         <is>
-          <t>1.038s</t>
+          <t>0.150s</t>
         </is>
       </c>
       <c r="O156" s="3" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>1.655s</t>
+          <t>1.503s</t>
         </is>
       </c>
       <c r="O157" s="3" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="N158" s="2" t="inlineStr">
         <is>
-          <t>1.357s</t>
+          <t>1.446s</t>
         </is>
       </c>
       <c r="O158" s="3" t="inlineStr">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="N159" s="2" t="inlineStr">
         <is>
-          <t>0.495s</t>
+          <t>0.079s</t>
         </is>
       </c>
       <c r="O159" s="3" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="N160" s="2" t="inlineStr">
         <is>
-          <t>1.405s</t>
+          <t>0.866s</t>
         </is>
       </c>
       <c r="O160" s="3" t="inlineStr">
@@ -16395,7 +16395,7 @@
       </c>
       <c r="N161" s="2" t="inlineStr">
         <is>
-          <t>1.187s</t>
+          <t>0.834s</t>
         </is>
       </c>
       <c r="O161" s="3" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="N162" s="2" t="inlineStr">
         <is>
-          <t>0.970s</t>
+          <t>1.532s</t>
         </is>
       </c>
       <c r="O162" s="3" t="inlineStr">
@@ -16593,7 +16593,7 @@
       </c>
       <c r="N163" s="2" t="inlineStr">
         <is>
-          <t>0.800s</t>
+          <t>0.412s</t>
         </is>
       </c>
       <c r="O163" s="3" t="inlineStr">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="N164" s="2" t="inlineStr">
         <is>
-          <t>0.967s</t>
+          <t>1.174s</t>
         </is>
       </c>
       <c r="O164" s="3" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="N165" s="2" t="inlineStr">
         <is>
-          <t>1.318s</t>
+          <t>1.355s</t>
         </is>
       </c>
       <c r="O165" s="3" t="inlineStr">
@@ -16890,7 +16890,7 @@
       </c>
       <c r="N166" s="2" t="inlineStr">
         <is>
-          <t>0.208s</t>
+          <t>1.274s</t>
         </is>
       </c>
       <c r="O166" s="3" t="inlineStr">
@@ -16989,7 +16989,7 @@
       </c>
       <c r="N167" s="2" t="inlineStr">
         <is>
-          <t>0.294s</t>
+          <t>1.242s</t>
         </is>
       </c>
       <c r="O167" s="3" t="inlineStr">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="N168" s="2" t="inlineStr">
         <is>
-          <t>0.571s</t>
+          <t>1.172s</t>
         </is>
       </c>
       <c r="O168" s="3" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="N169" s="2" t="inlineStr">
         <is>
-          <t>0.777s</t>
+          <t>1.442s</t>
         </is>
       </c>
       <c r="O169" s="3" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="N170" s="2" t="inlineStr">
         <is>
-          <t>1.606s</t>
+          <t>1.012s</t>
         </is>
       </c>
       <c r="O170" s="3" t="inlineStr">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="N171" s="2" t="inlineStr">
         <is>
-          <t>1.742s</t>
+          <t>0.948s</t>
         </is>
       </c>
       <c r="O171" s="3" t="inlineStr">
@@ -17484,7 +17484,7 @@
       </c>
       <c r="N172" s="2" t="inlineStr">
         <is>
-          <t>0.511s</t>
+          <t>0.503s</t>
         </is>
       </c>
       <c r="O172" s="3" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="N173" s="2" t="inlineStr">
         <is>
-          <t>1.530s</t>
+          <t>0.698s</t>
         </is>
       </c>
       <c r="O173" s="3" t="inlineStr">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="N174" s="2" t="inlineStr">
         <is>
-          <t>0.138s</t>
+          <t>0.492s</t>
         </is>
       </c>
       <c r="O174" s="3" t="inlineStr">
@@ -17781,7 +17781,7 @@
       </c>
       <c r="N175" s="2" t="inlineStr">
         <is>
-          <t>0.801s</t>
+          <t>0.151s</t>
         </is>
       </c>
       <c r="O175" s="3" t="inlineStr">
@@ -17880,7 +17880,7 @@
       </c>
       <c r="N176" s="2" t="inlineStr">
         <is>
-          <t>1.312s</t>
+          <t>1.558s</t>
         </is>
       </c>
       <c r="O176" s="3" t="inlineStr">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="N177" s="2" t="inlineStr">
         <is>
-          <t>0.173s</t>
+          <t>0.855s</t>
         </is>
       </c>
       <c r="O177" s="3" t="inlineStr">
@@ -18078,7 +18078,7 @@
       </c>
       <c r="N178" s="2" t="inlineStr">
         <is>
-          <t>1.006s</t>
+          <t>1.168s</t>
         </is>
       </c>
       <c r="O178" s="3" t="inlineStr">
@@ -18177,7 +18177,7 @@
       </c>
       <c r="N179" s="2" t="inlineStr">
         <is>
-          <t>0.158s</t>
+          <t>0.656s</t>
         </is>
       </c>
       <c r="O179" s="3" t="inlineStr">
@@ -18276,7 +18276,7 @@
       </c>
       <c r="N180" s="2" t="inlineStr">
         <is>
-          <t>1.844s</t>
+          <t>0.688s</t>
         </is>
       </c>
       <c r="O180" s="3" t="inlineStr">
@@ -18375,7 +18375,7 @@
       </c>
       <c r="N181" s="2" t="inlineStr">
         <is>
-          <t>0.130s</t>
+          <t>1.452s</t>
         </is>
       </c>
       <c r="O181" s="3" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="N182" s="2" t="inlineStr">
         <is>
-          <t>0.776s</t>
+          <t>1.506s</t>
         </is>
       </c>
       <c r="O182" s="3" t="inlineStr">
@@ -18573,7 +18573,7 @@
       </c>
       <c r="N183" s="2" t="inlineStr">
         <is>
-          <t>0.862s</t>
+          <t>1.606s</t>
         </is>
       </c>
       <c r="O183" s="3" t="inlineStr">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="N184" s="2" t="inlineStr">
         <is>
-          <t>0.473s</t>
+          <t>1.586s</t>
         </is>
       </c>
       <c r="O184" s="3" t="inlineStr">
@@ -18771,7 +18771,7 @@
       </c>
       <c r="N185" s="2" t="inlineStr">
         <is>
-          <t>0.225s</t>
+          <t>0.676s</t>
         </is>
       </c>
       <c r="O185" s="3" t="inlineStr">
@@ -18870,7 +18870,7 @@
       </c>
       <c r="N186" s="2" t="inlineStr">
         <is>
-          <t>0.592s</t>
+          <t>0.194s</t>
         </is>
       </c>
       <c r="O186" s="3" t="inlineStr">
@@ -18969,7 +18969,7 @@
       </c>
       <c r="N187" s="2" t="inlineStr">
         <is>
-          <t>1.138s</t>
+          <t>1.723s</t>
         </is>
       </c>
       <c r="O187" s="3" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="N188" s="2" t="inlineStr">
         <is>
-          <t>1.491s</t>
+          <t>0.253s</t>
         </is>
       </c>
       <c r="O188" s="3" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="N189" s="2" t="inlineStr">
         <is>
-          <t>1.267s</t>
+          <t>0.351s</t>
         </is>
       </c>
       <c r="O189" s="3" t="inlineStr">
@@ -19266,7 +19266,7 @@
       </c>
       <c r="N190" s="2" t="inlineStr">
         <is>
-          <t>0.084s</t>
+          <t>1.017s</t>
         </is>
       </c>
       <c r="O190" s="3" t="inlineStr">
@@ -19365,7 +19365,7 @@
       </c>
       <c r="N191" s="2" t="inlineStr">
         <is>
-          <t>1.806s</t>
+          <t>1.287s</t>
         </is>
       </c>
       <c r="O191" s="3" t="inlineStr">
@@ -19464,7 +19464,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>1.404s</t>
+          <t>1.767s</t>
         </is>
       </c>
       <c r="O192" s="3" t="inlineStr">
@@ -19563,7 +19563,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>0.284s</t>
+          <t>1.675s</t>
         </is>
       </c>
       <c r="O193" s="3" t="inlineStr">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>1.396s</t>
+          <t>0.410s</t>
         </is>
       </c>
       <c r="O194" s="3" t="inlineStr">
@@ -19761,7 +19761,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>0.373s</t>
+          <t>0.936s</t>
         </is>
       </c>
       <c r="O195" s="3" t="inlineStr">
@@ -19860,7 +19860,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>1.702s</t>
+          <t>0.797s</t>
         </is>
       </c>
       <c r="O196" s="3" t="inlineStr">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="N197" s="2" t="inlineStr">
         <is>
-          <t>0.962s</t>
+          <t>0.719s</t>
         </is>
       </c>
       <c r="O197" s="3" t="inlineStr">
@@ -20058,7 +20058,7 @@
       </c>
       <c r="N198" s="2" t="inlineStr">
         <is>
-          <t>1.115s</t>
+          <t>0.603s</t>
         </is>
       </c>
       <c r="O198" s="3" t="inlineStr">
@@ -20157,7 +20157,7 @@
       </c>
       <c r="N199" s="2" t="inlineStr">
         <is>
-          <t>0.640s</t>
+          <t>1.249s</t>
         </is>
       </c>
       <c r="O199" s="3" t="inlineStr">
@@ -20256,7 +20256,7 @@
       </c>
       <c r="N200" s="2" t="inlineStr">
         <is>
-          <t>0.346s</t>
+          <t>1.338s</t>
         </is>
       </c>
       <c r="O200" s="3" t="inlineStr">
@@ -20355,7 +20355,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>0.873s</t>
+          <t>0.346s</t>
         </is>
       </c>
       <c r="O201" s="3" t="inlineStr">
@@ -20454,7 +20454,7 @@
       </c>
       <c r="N202" s="2" t="inlineStr">
         <is>
-          <t>0.362s</t>
+          <t>0.654s</t>
         </is>
       </c>
       <c r="O202" s="3" t="inlineStr">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>1.331s</t>
+          <t>1.545s</t>
         </is>
       </c>
       <c r="O203" s="3" t="inlineStr">
@@ -20652,7 +20652,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>0.418s</t>
+          <t>1.199s</t>
         </is>
       </c>
       <c r="O204" s="3" t="inlineStr">
@@ -20751,7 +20751,7 @@
       </c>
       <c r="N205" s="2" t="inlineStr">
         <is>
-          <t>1.846s</t>
+          <t>1.742s</t>
         </is>
       </c>
       <c r="O205" s="3" t="inlineStr">
@@ -20850,7 +20850,7 @@
       </c>
       <c r="N206" s="2" t="inlineStr">
         <is>
-          <t>0.250s</t>
+          <t>1.529s</t>
         </is>
       </c>
       <c r="O206" s="3" t="inlineStr">
@@ -20949,7 +20949,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>1.167s</t>
+          <t>0.257s</t>
         </is>
       </c>
       <c r="O207" s="3" t="inlineStr">
@@ -21048,7 +21048,7 @@
       </c>
       <c r="N208" s="2" t="inlineStr">
         <is>
-          <t>1.011s</t>
+          <t>1.328s</t>
         </is>
       </c>
       <c r="O208" s="3" t="inlineStr">
@@ -21147,7 +21147,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>1.103s</t>
+          <t>0.064s</t>
         </is>
       </c>
       <c r="O209" s="3" t="inlineStr">
@@ -21246,7 +21246,7 @@
       </c>
       <c r="N210" s="2" t="inlineStr">
         <is>
-          <t>0.426s</t>
+          <t>1.406s</t>
         </is>
       </c>
       <c r="O210" s="3" t="inlineStr">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="N211" s="2" t="inlineStr">
         <is>
-          <t>0.604s</t>
+          <t>0.303s</t>
         </is>
       </c>
       <c r="O211" s="3" t="inlineStr">
@@ -21444,7 +21444,7 @@
       </c>
       <c r="N212" s="2" t="inlineStr">
         <is>
-          <t>0.797s</t>
+          <t>0.823s</t>
         </is>
       </c>
       <c r="O212" s="3" t="inlineStr">
@@ -21543,7 +21543,7 @@
       </c>
       <c r="N213" s="2" t="inlineStr">
         <is>
-          <t>1.433s</t>
+          <t>1.009s</t>
         </is>
       </c>
       <c r="O213" s="3" t="inlineStr">
@@ -21642,7 +21642,7 @@
       </c>
       <c r="N214" s="2" t="inlineStr">
         <is>
-          <t>1.848s</t>
+          <t>0.540s</t>
         </is>
       </c>
       <c r="O214" s="3" t="inlineStr">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="N215" s="2" t="inlineStr">
         <is>
-          <t>0.904s</t>
+          <t>0.807s</t>
         </is>
       </c>
       <c r="O215" s="3" t="inlineStr">
@@ -21840,7 +21840,7 @@
       </c>
       <c r="N216" s="2" t="inlineStr">
         <is>
-          <t>1.839s</t>
+          <t>1.108s</t>
         </is>
       </c>
       <c r="O216" s="3" t="inlineStr">
@@ -21939,7 +21939,7 @@
       </c>
       <c r="N217" s="2" t="inlineStr">
         <is>
-          <t>0.551s</t>
+          <t>0.189s</t>
         </is>
       </c>
       <c r="O217" s="3" t="inlineStr">
@@ -22038,7 +22038,7 @@
       </c>
       <c r="N218" s="2" t="inlineStr">
         <is>
-          <t>0.837s</t>
+          <t>1.699s</t>
         </is>
       </c>
       <c r="O218" s="3" t="inlineStr">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="N219" s="2" t="inlineStr">
         <is>
-          <t>1.177s</t>
+          <t>1.622s</t>
         </is>
       </c>
       <c r="O219" s="3" t="inlineStr">
@@ -22236,7 +22236,7 @@
       </c>
       <c r="N220" s="2" t="inlineStr">
         <is>
-          <t>0.635s</t>
+          <t>1.467s</t>
         </is>
       </c>
       <c r="O220" s="3" t="inlineStr">
@@ -22335,7 +22335,7 @@
       </c>
       <c r="N221" s="2" t="inlineStr">
         <is>
-          <t>0.784s</t>
+          <t>0.517s</t>
         </is>
       </c>
       <c r="O221" s="3" t="inlineStr">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="N222" s="2" t="inlineStr">
         <is>
-          <t>0.611s</t>
+          <t>1.712s</t>
         </is>
       </c>
       <c r="O222" s="3" t="inlineStr">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="N223" s="2" t="inlineStr">
         <is>
-          <t>0.728s</t>
+          <t>1.510s</t>
         </is>
       </c>
       <c r="O223" s="3" t="inlineStr">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="N224" s="2" t="inlineStr">
         <is>
-          <t>0.365s</t>
+          <t>0.311s</t>
         </is>
       </c>
       <c r="O224" s="3" t="inlineStr">
@@ -22731,7 +22731,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>1.599s</t>
+          <t>0.948s</t>
         </is>
       </c>
       <c r="O225" s="3" t="inlineStr">
@@ -22830,7 +22830,7 @@
       </c>
       <c r="N226" s="2" t="inlineStr">
         <is>
-          <t>1.813s</t>
+          <t>1.752s</t>
         </is>
       </c>
       <c r="O226" s="3" t="inlineStr">
@@ -22929,7 +22929,7 @@
       </c>
       <c r="N227" s="2" t="inlineStr">
         <is>
-          <t>0.698s</t>
+          <t>1.286s</t>
         </is>
       </c>
       <c r="O227" s="3" t="inlineStr">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="N228" s="2" t="inlineStr">
         <is>
-          <t>1.123s</t>
+          <t>1.453s</t>
         </is>
       </c>
       <c r="O228" s="3" t="inlineStr">
@@ -23127,7 +23127,7 @@
       </c>
       <c r="N229" s="2" t="inlineStr">
         <is>
-          <t>0.232s</t>
+          <t>0.956s</t>
         </is>
       </c>
       <c r="O229" s="3" t="inlineStr">
@@ -23226,7 +23226,7 @@
       </c>
       <c r="N230" s="2" t="inlineStr">
         <is>
-          <t>0.241s</t>
+          <t>0.116s</t>
         </is>
       </c>
       <c r="O230" s="3" t="inlineStr">
@@ -23325,7 +23325,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>0.639s</t>
+          <t>0.867s</t>
         </is>
       </c>
       <c r="O231" s="3" t="inlineStr">
@@ -23424,7 +23424,7 @@
       </c>
       <c r="N232" s="2" t="inlineStr">
         <is>
-          <t>1.215s</t>
+          <t>1.324s</t>
         </is>
       </c>
       <c r="O232" s="3" t="inlineStr">
@@ -23523,7 +23523,7 @@
       </c>
       <c r="N233" s="2" t="inlineStr">
         <is>
-          <t>1.598s</t>
+          <t>0.798s</t>
         </is>
       </c>
       <c r="O233" s="3" t="inlineStr">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="N234" s="2" t="inlineStr">
         <is>
-          <t>0.979s</t>
+          <t>1.043s</t>
         </is>
       </c>
       <c r="O234" s="3" t="inlineStr">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="N235" s="2" t="inlineStr">
         <is>
-          <t>1.164s</t>
+          <t>0.071s</t>
         </is>
       </c>
       <c r="O235" s="3" t="inlineStr">
@@ -23820,7 +23820,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>1.025s</t>
+          <t>1.275s</t>
         </is>
       </c>
       <c r="O236" s="3" t="inlineStr">
@@ -23919,7 +23919,7 @@
       </c>
       <c r="N237" s="2" t="inlineStr">
         <is>
-          <t>0.663s</t>
+          <t>1.745s</t>
         </is>
       </c>
       <c r="O237" s="3" t="inlineStr">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="N238" s="2" t="inlineStr">
         <is>
-          <t>1.346s</t>
+          <t>0.572s</t>
         </is>
       </c>
       <c r="O238" s="3" t="inlineStr">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="N239" s="2" t="inlineStr">
         <is>
-          <t>0.714s</t>
+          <t>1.668s</t>
         </is>
       </c>
       <c r="O239" s="3" t="inlineStr">
@@ -24216,7 +24216,7 @@
       </c>
       <c r="N240" s="2" t="inlineStr">
         <is>
-          <t>0.342s</t>
+          <t>1.223s</t>
         </is>
       </c>
       <c r="O240" s="3" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="N241" s="2" t="inlineStr">
         <is>
-          <t>0.533s</t>
+          <t>1.726s</t>
         </is>
       </c>
       <c r="O241" s="3" t="inlineStr">
@@ -24414,7 +24414,7 @@
       </c>
       <c r="N242" s="2" t="inlineStr">
         <is>
-          <t>1.654s</t>
+          <t>1.172s</t>
         </is>
       </c>
       <c r="O242" s="3" t="inlineStr">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="N243" s="2" t="inlineStr">
         <is>
-          <t>0.110s</t>
+          <t>1.332s</t>
         </is>
       </c>
       <c r="O243" s="3" t="inlineStr">
@@ -24612,7 +24612,7 @@
       </c>
       <c r="N244" s="2" t="inlineStr">
         <is>
-          <t>0.215s</t>
+          <t>0.413s</t>
         </is>
       </c>
       <c r="O244" s="3" t="inlineStr">
@@ -24711,7 +24711,7 @@
       </c>
       <c r="N245" s="2" t="inlineStr">
         <is>
-          <t>0.885s</t>
+          <t>0.398s</t>
         </is>
       </c>
       <c r="O245" s="3" t="inlineStr">
@@ -24810,7 +24810,7 @@
       </c>
       <c r="N246" s="2" t="inlineStr">
         <is>
-          <t>0.230s</t>
+          <t>1.359s</t>
         </is>
       </c>
       <c r="O246" s="3" t="inlineStr">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="N247" s="2" t="inlineStr">
         <is>
-          <t>0.755s</t>
+          <t>1.491s</t>
         </is>
       </c>
       <c r="O247" s="3" t="inlineStr">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="N248" s="2" t="inlineStr">
         <is>
-          <t>1.740s</t>
+          <t>1.144s</t>
         </is>
       </c>
       <c r="O248" s="3" t="inlineStr">
@@ -25107,7 +25107,7 @@
       </c>
       <c r="N249" s="2" t="inlineStr">
         <is>
-          <t>0.661s</t>
+          <t>1.072s</t>
         </is>
       </c>
       <c r="O249" s="3" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="N250" s="2" t="inlineStr">
         <is>
-          <t>0.949s</t>
+          <t>0.628s</t>
         </is>
       </c>
       <c r="O250" s="3" t="inlineStr">
@@ -25305,7 +25305,7 @@
       </c>
       <c r="N251" s="2" t="inlineStr">
         <is>
-          <t>0.910s</t>
+          <t>0.827s</t>
         </is>
       </c>
       <c r="O251" s="3" t="inlineStr">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="N252" s="2" t="inlineStr">
         <is>
-          <t>0.428s</t>
+          <t>1.559s</t>
         </is>
       </c>
       <c r="O252" s="3" t="inlineStr">
@@ -25503,7 +25503,7 @@
       </c>
       <c r="N253" s="2" t="inlineStr">
         <is>
-          <t>1.100s</t>
+          <t>0.805s</t>
         </is>
       </c>
       <c r="O253" s="3" t="inlineStr">
@@ -25602,7 +25602,7 @@
       </c>
       <c r="N254" s="2" t="inlineStr">
         <is>
-          <t>0.541s</t>
+          <t>0.499s</t>
         </is>
       </c>
       <c r="O254" s="3" t="inlineStr">
@@ -25701,7 +25701,7 @@
       </c>
       <c r="N255" s="2" t="inlineStr">
         <is>
-          <t>1.080s</t>
+          <t>1.731s</t>
         </is>
       </c>
       <c r="O255" s="3" t="inlineStr">
@@ -25800,7 +25800,7 @@
       </c>
       <c r="N256" s="2" t="inlineStr">
         <is>
-          <t>1.361s</t>
+          <t>1.187s</t>
         </is>
       </c>
       <c r="O256" s="3" t="inlineStr">
@@ -25899,7 +25899,7 @@
       </c>
       <c r="N257" s="2" t="inlineStr">
         <is>
-          <t>1.256s</t>
+          <t>0.212s</t>
         </is>
       </c>
       <c r="O257" s="3" t="inlineStr">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="N258" s="2" t="inlineStr">
         <is>
-          <t>1.709s</t>
+          <t>1.483s</t>
         </is>
       </c>
       <c r="O258" s="3" t="inlineStr">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="N259" s="2" t="inlineStr">
         <is>
-          <t>0.343s</t>
+          <t>0.480s</t>
         </is>
       </c>
       <c r="O259" s="3" t="inlineStr">
@@ -26196,7 +26196,7 @@
       </c>
       <c r="N260" s="2" t="inlineStr">
         <is>
-          <t>1.537s</t>
+          <t>1.520s</t>
         </is>
       </c>
       <c r="O260" s="3" t="inlineStr">
@@ -26295,7 +26295,7 @@
       </c>
       <c r="N261" s="2" t="inlineStr">
         <is>
-          <t>1.508s</t>
+          <t>1.017s</t>
         </is>
       </c>
       <c r="O261" s="3" t="inlineStr">
@@ -26394,7 +26394,7 @@
       </c>
       <c r="N262" s="2" t="inlineStr">
         <is>
-          <t>1.525s</t>
+          <t>1.672s</t>
         </is>
       </c>
       <c r="O262" s="3" t="inlineStr">
@@ -26493,7 +26493,7 @@
       </c>
       <c r="N263" s="2" t="inlineStr">
         <is>
-          <t>1.832s</t>
+          <t>1.033s</t>
         </is>
       </c>
       <c r="O263" s="3" t="inlineStr">
@@ -26592,7 +26592,7 @@
       </c>
       <c r="N264" s="2" t="inlineStr">
         <is>
-          <t>0.175s</t>
+          <t>1.622s</t>
         </is>
       </c>
       <c r="O264" s="3" t="inlineStr">
@@ -26691,7 +26691,7 @@
       </c>
       <c r="N265" s="2" t="inlineStr">
         <is>
-          <t>0.603s</t>
+          <t>0.332s</t>
         </is>
       </c>
       <c r="O265" s="3" t="inlineStr">
@@ -26790,7 +26790,7 @@
       </c>
       <c r="N266" s="2" t="inlineStr">
         <is>
-          <t>0.162s</t>
+          <t>1.298s</t>
         </is>
       </c>
       <c r="O266" s="3" t="inlineStr">
@@ -26889,7 +26889,7 @@
       </c>
       <c r="N267" s="2" t="inlineStr">
         <is>
-          <t>1.665s</t>
+          <t>0.876s</t>
         </is>
       </c>
       <c r="O267" s="3" t="inlineStr">
@@ -26988,7 +26988,7 @@
       </c>
       <c r="N268" s="2" t="inlineStr">
         <is>
-          <t>1.399s</t>
+          <t>1.510s</t>
         </is>
       </c>
       <c r="O268" s="3" t="inlineStr">
@@ -27087,7 +27087,7 @@
       </c>
       <c r="N269" s="2" t="inlineStr">
         <is>
-          <t>0.678s</t>
+          <t>1.556s</t>
         </is>
       </c>
       <c r="O269" s="3" t="inlineStr">
@@ -27186,7 +27186,7 @@
       </c>
       <c r="N270" s="2" t="inlineStr">
         <is>
-          <t>0.980s</t>
+          <t>1.153s</t>
         </is>
       </c>
       <c r="O270" s="3" t="inlineStr">
@@ -27285,7 +27285,7 @@
       </c>
       <c r="N271" s="2" t="inlineStr">
         <is>
-          <t>0.678s</t>
+          <t>1.127s</t>
         </is>
       </c>
       <c r="O271" s="3" t="inlineStr">
@@ -27384,7 +27384,7 @@
       </c>
       <c r="N272" s="2" t="inlineStr">
         <is>
-          <t>0.444s</t>
+          <t>0.674s</t>
         </is>
       </c>
       <c r="O272" s="3" t="inlineStr">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="N273" s="2" t="inlineStr">
         <is>
-          <t>0.197s</t>
+          <t>0.316s</t>
         </is>
       </c>
       <c r="O273" s="3" t="inlineStr">
@@ -27582,7 +27582,7 @@
       </c>
       <c r="N274" s="2" t="inlineStr">
         <is>
-          <t>0.955s</t>
+          <t>1.445s</t>
         </is>
       </c>
       <c r="O274" s="3" t="inlineStr">
@@ -27681,7 +27681,7 @@
       </c>
       <c r="N275" s="2" t="inlineStr">
         <is>
-          <t>0.406s</t>
+          <t>1.385s</t>
         </is>
       </c>
       <c r="O275" s="3" t="inlineStr">
@@ -27780,7 +27780,7 @@
       </c>
       <c r="N276" s="2" t="inlineStr">
         <is>
-          <t>1.120s</t>
+          <t>1.430s</t>
         </is>
       </c>
       <c r="O276" s="3" t="inlineStr">
@@ -27879,7 +27879,7 @@
       </c>
       <c r="N277" s="2" t="inlineStr">
         <is>
-          <t>1.093s</t>
+          <t>1.385s</t>
         </is>
       </c>
       <c r="O277" s="3" t="inlineStr">
@@ -27978,7 +27978,7 @@
       </c>
       <c r="N278" s="2" t="inlineStr">
         <is>
-          <t>1.836s</t>
+          <t>1.292s</t>
         </is>
       </c>
       <c r="O278" s="3" t="inlineStr">
@@ -28077,7 +28077,7 @@
       </c>
       <c r="N279" s="2" t="inlineStr">
         <is>
-          <t>1.427s</t>
+          <t>0.769s</t>
         </is>
       </c>
       <c r="O279" s="3" t="inlineStr">
@@ -28176,7 +28176,7 @@
       </c>
       <c r="N280" s="2" t="inlineStr">
         <is>
-          <t>0.693s</t>
+          <t>0.878s</t>
         </is>
       </c>
       <c r="O280" s="3" t="inlineStr">
@@ -28275,7 +28275,7 @@
       </c>
       <c r="N281" s="2" t="inlineStr">
         <is>
-          <t>0.083s</t>
+          <t>1.827s</t>
         </is>
       </c>
       <c r="O281" s="3" t="inlineStr">
@@ -28374,7 +28374,7 @@
       </c>
       <c r="N282" s="2" t="inlineStr">
         <is>
-          <t>0.564s</t>
+          <t>0.535s</t>
         </is>
       </c>
       <c r="O282" s="3" t="inlineStr">
@@ -28473,7 +28473,7 @@
       </c>
       <c r="N283" s="2" t="inlineStr">
         <is>
-          <t>1.265s</t>
+          <t>0.981s</t>
         </is>
       </c>
       <c r="O283" s="3" t="inlineStr">
@@ -28572,7 +28572,7 @@
       </c>
       <c r="N284" s="2" t="inlineStr">
         <is>
-          <t>0.247s</t>
+          <t>0.595s</t>
         </is>
       </c>
       <c r="O284" s="3" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="N285" s="2" t="inlineStr">
         <is>
-          <t>0.071s</t>
+          <t>0.845s</t>
         </is>
       </c>
       <c r="O285" s="3" t="inlineStr">
@@ -28770,7 +28770,7 @@
       </c>
       <c r="N286" s="2" t="inlineStr">
         <is>
-          <t>0.740s</t>
+          <t>1.740s</t>
         </is>
       </c>
       <c r="O286" s="3" t="inlineStr">
@@ -28869,7 +28869,7 @@
       </c>
       <c r="N287" s="2" t="inlineStr">
         <is>
-          <t>0.077s</t>
+          <t>0.655s</t>
         </is>
       </c>
       <c r="O287" s="3" t="inlineStr">
@@ -28968,7 +28968,7 @@
       </c>
       <c r="N288" s="2" t="inlineStr">
         <is>
-          <t>1.515s</t>
+          <t>0.227s</t>
         </is>
       </c>
       <c r="O288" s="3" t="inlineStr">
@@ -29067,7 +29067,7 @@
       </c>
       <c r="N289" s="2" t="inlineStr">
         <is>
-          <t>1.610s</t>
+          <t>1.548s</t>
         </is>
       </c>
       <c r="O289" s="3" t="inlineStr">
@@ -29166,7 +29166,7 @@
       </c>
       <c r="N290" s="2" t="inlineStr">
         <is>
-          <t>1.481s</t>
+          <t>0.343s</t>
         </is>
       </c>
       <c r="O290" s="3" t="inlineStr">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="N291" s="2" t="inlineStr">
         <is>
-          <t>0.179s</t>
+          <t>1.438s</t>
         </is>
       </c>
       <c r="O291" s="3" t="inlineStr">
@@ -29364,7 +29364,7 @@
       </c>
       <c r="N292" s="2" t="inlineStr">
         <is>
-          <t>0.854s</t>
+          <t>1.636s</t>
         </is>
       </c>
       <c r="O292" s="3" t="inlineStr">
@@ -29463,7 +29463,7 @@
       </c>
       <c r="N293" s="2" t="inlineStr">
         <is>
-          <t>0.446s</t>
+          <t>0.097s</t>
         </is>
       </c>
       <c r="O293" s="3" t="inlineStr">
@@ -29562,7 +29562,7 @@
       </c>
       <c r="N294" s="2" t="inlineStr">
         <is>
-          <t>0.522s</t>
+          <t>1.253s</t>
         </is>
       </c>
       <c r="O294" s="3" t="inlineStr">
@@ -29661,7 +29661,7 @@
       </c>
       <c r="N295" s="2" t="inlineStr">
         <is>
-          <t>1.123s</t>
+          <t>1.647s</t>
         </is>
       </c>
       <c r="O295" s="3" t="inlineStr">
@@ -29760,7 +29760,7 @@
       </c>
       <c r="N296" s="2" t="inlineStr">
         <is>
-          <t>0.861s</t>
+          <t>1.412s</t>
         </is>
       </c>
       <c r="O296" s="3" t="inlineStr">
@@ -29859,7 +29859,7 @@
       </c>
       <c r="N297" s="2" t="inlineStr">
         <is>
-          <t>0.288s</t>
+          <t>1.665s</t>
         </is>
       </c>
       <c r="O297" s="3" t="inlineStr">
@@ -29958,7 +29958,7 @@
       </c>
       <c r="N298" s="2" t="inlineStr">
         <is>
-          <t>1.725s</t>
+          <t>1.663s</t>
         </is>
       </c>
       <c r="O298" s="3" t="inlineStr">
@@ -30057,7 +30057,7 @@
       </c>
       <c r="N299" s="2" t="inlineStr">
         <is>
-          <t>1.497s</t>
+          <t>0.114s</t>
         </is>
       </c>
       <c r="O299" s="3" t="inlineStr">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="N300" s="2" t="inlineStr">
         <is>
-          <t>0.578s</t>
+          <t>0.427s</t>
         </is>
       </c>
       <c r="O300" s="3" t="inlineStr">
@@ -30255,7 +30255,7 @@
       </c>
       <c r="N301" s="2" t="inlineStr">
         <is>
-          <t>1.297s</t>
+          <t>1.732s</t>
         </is>
       </c>
       <c r="O301" s="3" t="inlineStr">

</xml_diff>